<commit_message>
Drop-and-play settings: optional Scope Settings sheet and a guided Setup page
A workbook can now carry a fifth sheet, Scope Settings, holding what the four
input sheets do not: investor display names, groups and attribution weights,
view definitions, fund look-through entered per investor, and the FX exception.
Every drop of that workbook is configured automatically; changes made in the
app take precedence and can be downloaded back into the sheet.

Data > Setup walks through loading, columns, investors, views, an investors x
funds look-through grid and the workbook checks. Workbooks can keep their
formulas: saved results are read, and formula columns that failed in the
workbook (e.g. references to sheets not exported) are skipped by the checks
instead of being reported as differences. Includes a test workbook with live
formulas.
</commit_message>
<xml_diff>
--- a/data/demo/Scope-demo.xlsx
+++ b/data/demo/Scope-demo.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Mapping" sheetId="2" r:id="rId2"/>
     <sheet name="Hardcoded" sheetId="3" r:id="rId3"/>
     <sheet name="ESG Hardcoded" sheetId="4" r:id="rId4"/>
+    <sheet name="Scope Settings" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -99006,4 +99007,635 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:V15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Scope Settings: names, groups and weights of investor columns, view definitions, fund look-through and the FX exception. Optional sheet; read by name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Investors</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Views</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Look Through</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>FX Exception</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Investor Column</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Display Name</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Attribution Weight</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Investor Column</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Investor 1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Group entity</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Total platform</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>All investors</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Investor 1</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="M4">
+        <v>0.15</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Investor 5</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Platform Beta</t>
+        </is>
+      </c>
+      <c r="R4">
+        <v>0.86</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>hedged rate for one investor on one view (synthetic example)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Attribution label</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Investor 2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Group entity</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Group (attributed)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Group weights</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Investor 3</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="M5">
+        <v>0.1</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>IG threshold</t>
+        </is>
+      </c>
+      <c r="V5">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Investor 3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Group entity</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Platform Alpha</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Investor 1</t>
+        </is>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Investor 5</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="M6">
+        <v>0.1</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Base currency</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Investor 4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Group entity</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Platform Alpha</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Investor 2</t>
+        </is>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Investor 9</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="M7">
+        <v>0.25</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>FX quote</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Investor 5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Group entity</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Platform Alpha</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Investor 3</t>
+        </is>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Investor 2</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Investor 8</t>
+        </is>
+      </c>
+      <c r="M8">
+        <v>0.12</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Single portfolio token</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>SINGLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Investor 6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Group entity</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Platform Alpha</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Investor 4</t>
+        </is>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Investor 6</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Investor 8</t>
+        </is>
+      </c>
+      <c r="M9">
+        <v>0.08</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Maturity buckets</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0-3, 3-5, 5-10, 10-20, 20+</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="E10">
+        <v>0.35</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Platform Beta</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Investor 5</t>
+        </is>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Investor 10</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Investor 8</t>
+        </is>
+      </c>
+      <c r="M10">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Investor 8</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="E11">
+        <v>0.2</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Platform Beta</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Investor 6</t>
+        </is>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Investor 9</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Third party</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Platform Beta</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Investor 10</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Third party</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Fund I look-through (35%)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Investor 7</t>
+        </is>
+      </c>
+      <c r="I13">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Investor 11</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Third party</t>
+        </is>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Investors 11+12</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Investor 11</t>
+        </is>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Investor 12</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Third party</t>
+        </is>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Investors 11+12</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Investor 12</t>
+        </is>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>